<commit_message>
Make the roll-call header fields easier to fill in.
Date, time, person in charge, and place now sit in bordered boxes that are wide enough to write in.

Co-authored-by: kayeekelly722 <kayeekelly722@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/船河樂2026_點名表.xlsx
+++ b/船河樂2026_點名表.xlsx
@@ -154,7 +154,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E7EEF4"/>
+        <fgColor rgb="00F8F1DE"/>
       </patternFill>
     </fill>
     <fill>
@@ -246,27 +246,27 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00E7EEF4"/>
+        <color rgb="00F8F1DE"/>
       </left>
       <right style="thin">
-        <color rgb="00E7EEF4"/>
+        <color rgb="00F8F1DE"/>
       </right>
       <top style="thin">
-        <color rgb="00E7EEF4"/>
+        <color rgb="00F8F1DE"/>
       </top>
       <bottom style="thin">
-        <color rgb="00E7EEF4"/>
+        <color rgb="00F8F1DE"/>
       </bottom>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00E7EEF4"/>
+      <left style="medium">
+        <color rgb="001B4F72"/>
       </left>
-      <right style="thin">
-        <color rgb="00E7EEF4"/>
+      <right style="medium">
+        <color rgb="001B4F72"/>
       </right>
-      <top style="thin">
-        <color rgb="00E7EEF4"/>
+      <top style="medium">
+        <color rgb="001B4F72"/>
       </top>
       <bottom style="medium">
         <color rgb="001B4F72"/>
@@ -411,7 +411,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1069,7 +1069,7 @@
       <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="n"/>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>日期</t>
@@ -1085,20 +1085,20 @@
       <c r="E3" s="3" t="n"/>
       <c r="F3" s="4" t="n"/>
       <c r="G3" s="4" t="n"/>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>負責人</t>
         </is>
       </c>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="4" t="n"/>
+      <c r="J3" s="3" t="n"/>
       <c r="K3" s="4" t="n"/>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="L3" s="4" t="n"/>
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>地點</t>
         </is>
       </c>
-      <c r="M3" s="4" t="n"/>
       <c r="N3" s="4" t="n"/>
       <c r="O3" s="4" t="n"/>
     </row>
@@ -2675,23 +2675,23 @@
   <mergeCells count="19">
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="J4:L4"/>
-    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="N3:O3"/>
     <mergeCell ref="A2:O2"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="G5:I5"/>
     <mergeCell ref="D4:F4"/>
-    <mergeCell ref="M3:O3"/>
     <mergeCell ref="G4:I4"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="I3:J3"/>
     <mergeCell ref="D5:F5"/>
     <mergeCell ref="M4:O4"/>
     <mergeCell ref="D3:E3"/>
-    <mergeCell ref="H3:I3"/>
     <mergeCell ref="J5:L5"/>
-    <mergeCell ref="J3:K3"/>
     <mergeCell ref="M5:O5"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A1:O1"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="K3:L3"/>
   </mergeCells>
   <conditionalFormatting sqref="N7:N27">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">

</xml_diff>